<commit_message>
Add gated-asset scoring pipeline and dashboard tab, update README
- build_gated_content.py: manual capture of real PDF text for the 26
  gated whitepapers/eBooks pulled from SharePoint (JS-gated HubSpot
  forms extract_content.py can't reach on its own)
- score_gated_assets.py: separate 5-axis sales-enablement rubric
  (accuracy, brand, sales usability, substance, next-step clarity) --
  deliberately not the SEO/conversion rubric, since these PDFs aren't
  found via search
- combine_workbook.py: merges both scoring runs into one two-sheet
  workbook (Marketing Surface + Gated Asset Quality)
- build_site.py: reads the two-sheet workbook, writes a JSON/CSV pair
  per sheet
- site/index.html: adds the missing piece -- a tab UI so the gated
  scores are actually reachable on the dashboard, config-driven so
  each tab renders its own score axes
- README: documents the actual current architecture end to end
</commit_message>
<xml_diff>
--- a/data/scored_2026-Q3.xlsx
+++ b/data/scored_2026-Q3.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing Surface" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gated Asset Quality" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -37159,4 +37160,2024 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Accuracy Score</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Brand Score</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Sales Usability Score</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Substance Score</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Next Step Score</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Composite Score</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Action Flag</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Suggestions</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Effort</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Last Audited</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/why-centralized-security-is-necessary/</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A Single Pane of Glass: Why Centralized Security is Necessary</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sales2/SALES Main Folder/Content/Whitepapers/Whitepaper - A Single Pane of Glass (Why centralizing security is necessary).pdf</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F2" t="n">
+        <v>11</v>
+      </c>
+      <c r="G2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>49</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>The biggest weakness is severe thinness and an absent call to action — the document ends abruptly with a one-sentence summary and no next step, making it essentially unusable as a standalone sales asset. Its biggest strength is the two concrete customer proof points (Sage Realty and Pepsi G&amp;J), which are credible and specific, but they carry the entire document.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>- Add a clear, explicit call to action at the close of the document — at minimum a line directing the reader to schedule a demo or contact sales at getgenea.com, since the document currently ends with a generic summary sentence and gives a converted prospect nowhere to go next; this is the single highest-impact fix for deal usability.
+- Replace the Cisco Meraki video management reference in the Pepsi G&amp;J case study with one of the VMS integrations documented in the current help center (Eagle Eye, Milestone Mobile Server, Milestone Kite, Tyco Cloud, or Arcules) — or verify Cisco Meraki is still a supported integration — because the help center reference articles provided show no Cisco Meraki integration, and a rep sending this to a prospect whose VMS is one of the documented platforms will look uninformed.
+- Expand the 'Centralizing Your Security' and 'The Solution to Disparate Systems' sections from thin assertions into a genuine framework — for example, a step-by-step evaluation checklist or a before/after workflow diagram showing how siloed systems consolidate into a single pane of glass — because as written these sections add almost no value a prospect couldn't get from a blog post, which undercuts the justification for gating the asset.
+- Add a current integration ecosystem section that names and briefly describes two or three of Genea's documented VMS integrations (e.g., Eagle Eye, Arcules, Milestone) with the camera-to-door mapping and instant video feed features described in the help center articles, turning an abstract claim about integrations into concrete proof of the 'single pane of glass' promise.
+- Remove or update the branding inconsistency — the document uses 'Genea Security' as the company name in the header while the domain is getgenea.com; confirm the current preferred brand name and apply it consistently, as a rep handing this to a prospect at a named-account deal should not have to explain a naming discrepancy.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/access-control-software-takeover/</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Access Control Software Takeover</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Sales2/SALES Main Folder/Content/One Sheets/Access Control Takover One Sheet.pdf (one-page one-sheet, not a full whitepaper)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" t="n">
+        <v>53</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>The biggest weakness is that this one-sheet is substantively thin for a gated asset — three generic bullet points and an unextracted logo list do not justify a form fill, and the document has no call to action whatsoever inside the content itself. Its biggest strength is that the core Mercury Takeover concept is accurate and well-aligned with Genea's non-proprietary hardware positioning as confirmed by the help center reference on Mercury MP vs LP series.</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>- Add a specific, clickable or printed call to action inside the document itself (e.g., 'Schedule a free Mercury Takeover assessment at getgenea.com/demo') — as filed, there is zero next-step guidance for the reader, which wastes every conversion this asset drives.
+- Replace the unextracted logo/system list with actual text naming the supported legacy systems (e.g., Lenel, Avigilon, Genetec, ACRE are cited in the help article 'Mercury MP series versus LP series' as Mercury-based platforms) so a prospect or rep reading a PDF copy knows at a glance whether their system qualifies without needing a rendered image.
+- Expand the one-sheet to address the controller replacement workflow described in the help article 'How to Replace a Mercury Controller in Genea,' specifically calling out that existing configurations and device associations are preserved during a takeover — this is the #1 customer anxiety and the doc never addresses it.
+- Quantify the cost savings claim: 'less expensive than you think' and 'save on capital expenditure' are vague; add even a directional figure (e.g., 'customers typically save X% vs. full hardware replacement') or a brief before/after scenario to give a rep something concrete to anchor a conversation.
+- Clarify that the takeover applies to the Mercury controller layer specifically (master controller reconfiguration) and note that sub-devices such as readers and credentials are also retained where compatible, drawing on the EP-to-LP/MP upgrade context in the help article 'How to Replace a Mercury Controller in Genea,' so prospects with mixed hardware don't self-disqualify incorrectly.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Quick Win</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/access-control-for-class-a-office-buildings/</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Access Control For Class A Office Buildings</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/Whitepapers/Access Control for Class A Office Buildings.pdf</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>13</v>
+      </c>
+      <c r="E4" t="n">
+        <v>14</v>
+      </c>
+      <c r="F4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" t="n">
+        <v>52</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>The document's most critical failure is that it has no call to action whatsoever — it ends abruptly mid-argument with no next step for the reader — making it nearly unusable as a standalone sales asset. Its biggest strength is that its core positioning (cloud vs. on-prem, non-proprietary Mercury hardware, open API) still aligns with Genea's current differentiation, but the content is extremely thin for a gated whitepaper.</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>- Add a closing call-to-action page or section directing the reader to schedule a demo at getgenea.com or contact their Genea rep — the document currently ends on a declarative statement with zero next-step instruction, which means every rep who sends this must manually follow up with guidance they should not have to provide.
+- Substantially expand the substance of the document: the entire asset is roughly 200 words and reads like a one-page leave-behind, not a whitepaper — add at minimum a worked cost-comparison example (e.g., contrasting TCO of a proprietary on-prem system vs. Genea over a 3-year contract), a tenant-experience scenario, or anonymized case data to justify the lead-capture friction.
+- Revise the Building Sync description ('enables tenants to add and remove employee keys from the access control system automatically') to accurately reflect the current product scope per the help article 'Building Sync - Building Administrator's Guide,' which clarifies that Building Sync keeps the building administrator's system in sync with the tenant's Genea access control system — the whitepaper's phrasing implies tenants self-manage keys in isolation, omitting the building-admin role and the requirement that the tenant suite also run Genea.
+- Add a video management / integrated security section referencing Genea's current VMS integrations (Milestone, Rhombus, Tyco Cloud) as documented in the help center — these integrations are directly relevant to Class A building risk management and operating efficiency claims made in the document but are completely absent, leaving a credibility gap for security-conscious prospects.
+- Replace or remove the dated tenant-app examples (HQO, Rise, Lane) with a current, verified integration list, or omit specific app names entirely if they cannot be confirmed as active — stale partner references are a liability when a prospect or their broker checks and finds a defunct or changed partnership.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/5-key-elements-for-a-touchless-access-control-building/</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>5 Key Elements for a Touchless Access Control Building</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/Whitepapers/5 Key Elements for a Touchless Access Control Building.pdf</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" t="n">
+        <v>11</v>
+      </c>
+      <c r="F5" t="n">
+        <v>9</v>
+      </c>
+      <c r="G5" t="n">
+        <v>7</v>
+      </c>
+      <c r="H5" t="n">
+        <v>13</v>
+      </c>
+      <c r="I5" t="n">
+        <v>48</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>The biggest issue is that the entire framing is anchored in COVID-19 as a present-tense business driver, which is severely dated and will undermine credibility with any prospect reading it today; the biggest strength is that the five-element structure maps reasonably well to real Genea capabilities (cloud platform, mobile credentials, visitor pre-registration, home-floor/DD integration, tenant education) that are confirmed by current help center documentation.</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>- Remove all COVID-19 framing entirely — phrases like 'While the world is dealing with the fallout of Covid-19' and 'daily occupancy is at all-time lows' will immediately signal to a prospect that this asset is stale and cause a rep to lose credibility; replace the opening with a current, evergreen business driver such as reducing front-desk overhead, improving tenant experience in a competitive leasing market, or supporting hybrid work models.
+- Expand Element 4 (destination dispatch / home-floor assignments for guests) using the current product detail confirmed in the help article 'Visitor Access to Home Floors' — specifically, add that visitors receive credentials in advance, swipe at the building entrance, and the DD system automatically assigns the correct elevator floor, which is a concrete and differentiating workflow the document currently describes only in a single vague sentence.
+- Add a substantive section or callout on Building Sync as a sixth element or expansion of Element 1, drawing on the help article 'Building Sync - Building Administrator's Guide' and 'How does check-in flow work with building sync?' — the document never mentions Building Sync by name, missing a key differentiator that eliminates admin overhead for tenant employee/card management and bridges building and tenant visitor management systems.
+- Flesh out each of the five elements from their current one-to-two sentence summaries into genuine frameworks with decision criteria, implementation considerations, or buyer questions to ask — as written, none of the five elements contains more depth than a blog post bullet point, which does not justify the friction of a lead-capture form fill.
+- Update the call to action to reference Genea's combined access control and visitor management platform by its current positioning language ('cloud-native,' 'non-proprietary hardware') rather than the generic phrase 'easy-to-use, cloud-based platform,' and add a secondary next step such as a relevant case study or related resource so reps have a follow-on send option.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/all-you-need-to-know-about-submetering/</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>All You Need to Know About Submetering</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/Whitepapers/All You Need to Know About Submetering- Whitepaper.pdf (modified Dec 2025)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E6" t="n">
+        <v>13</v>
+      </c>
+      <c r="F6" t="n">
+        <v>11</v>
+      </c>
+      <c r="G6" t="n">
+        <v>8</v>
+      </c>
+      <c r="H6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I6" t="n">
+        <v>52</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>The whitepaper is extremely thin — it reads as a short blog outline rather than a gated asset, offering almost no frameworks, data, or worked examples to justify a form fill; the biggest strength is that it is topically accurate at a high level and does not contradict the help center references, but it omits multiple current product capabilities (mobile app QR-code meter reading, Utility Bill Upload, metering statements) that the help center confirms exist today and would meaningfully deepen the content.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>- Expand the body with a concrete walkthrough of the end-to-end workflow using Genea's current product features — per the help articles 'How to Read a Meter?' and 'Getting Started with Genea's Submeter Billing Mobile App,' the QR-code scan → photo → confirm reading flow is a genuine differentiator that should be illustrated with a step-by-step example or screenshot to give the asset the depth that justifies gating it.
+- Add a section describing the Utility Bill Upload feature (per the help article 'Utility Bill Upload') — the ability to upload, review, and reconcile utility bills directly from the Invoicing page with a Utility Bill History tab is a concrete, current capability completely absent from the whitepaper that directly addresses the 'accounting for expenses' and 'accurate tenant billing' bullets already listed.
+- Replace the vague closing bullet list ('Accounting for Expenses, Accurate Tenant Billing…') with a clear, explicit call to action inside the document itself — e.g., 'Schedule a demo to see how Genea automates your submeter billing end to end at getgenea.com/demo' — since the document currently ends with no directional next step for the prospect.
+- Flesh out the RUBS vs. submetering comparison into a decision framework (e.g., a simple table showing cost thresholds, building types, and regulatory contexts where each approach is appropriate) so a prospect gets a defensible rationale they cannot find on a blog post, making the gated friction worthwhile.
+- Add at least one real or representative customer outcome (e.g., 'a mid-size commercial property reduced utility reconciliation time by X%') to support the cost-reduction and ESG claims — right now every benefit claim is asserted without evidence, which weakens credibility in a live deal context.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/resources-whitepapers-cloud-vs-on-prem-access-control-guide/</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Cloud vs On-Prem Access Control - Decision Guide</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Marketing/DEMAND GEN/Campaign Assets/Modernization in Motion_Q2 2026/Guide - Cloud vs On-Prem Access Control.pdf (modified Jun 2026 -- newest gated asset found)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>16</v>
+      </c>
+      <c r="E7" t="n">
+        <v>17</v>
+      </c>
+      <c r="F7" t="n">
+        <v>15</v>
+      </c>
+      <c r="G7" t="n">
+        <v>13</v>
+      </c>
+      <c r="H7" t="n">
+        <v>10</v>
+      </c>
+      <c r="I7" t="n">
+        <v>71</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Optimize</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>The biggest weakness is the 18-question diagnostic, which is described but never actually included in the document — a prospect who fills out a form to get a decision framework and finds the core tool missing will feel misled, which actively harms the deal. The biggest strength is the myth-busting structure, which is credible, balanced (acknowledging on-prem legitimacy), and aligned with Genea's open-hardware, non-lock-in positioning.</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>- Include the actual 18 diagnostic questions in the document — the guide promises 'a diagnostic: 18 questions' across five dimensions but delivers none of them, leaving the gated asset's core value proposition completely unfulfilled and forcing the rep to apologize or over-explain what the prospect is looking at.
+- Add a concrete next-step call to action beyond a passive reference to 'Genea's Migration Readiness Checklist' — the 'What to Do Next' section never links to, embeds, or offers a demo/contact path, so a motivated prospect who finishes reading has no clear way to engage Genea directly from this asset.
+- Expand the 'How Genea Approaches This' section with at least one specific integration example drawn from the actual product (e.g., the Assa Abloy Aperio wireless lock integration or Schlage AD/Engage series — both documented in current help articles — illustrate the open-hardware claim concretely rather than leaving it as a bullet point assertion).
+- Clarify the Mercury hardware claim by distinguishing MP vs LP series where relevant — the help article 'Mercury MP series versus LP series' shows Genea supports both lines with different use cases, and a prospect evaluating enterprise scalability would benefit from knowing this rather than seeing 'Mercury hardware' cited as a monolithic proof point.
+- Fix the malformed title on the cover page ('The Honest Guide to A decision framework for security and IT leaders') — the broken sentence reads as a production error and will make any rep pause before forwarding this to a CISO or VP of IT.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/driving-value-with-process-automation/</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Driving Value with Process Automation</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/eBooks/eBook - Driving Value with Process Automation.pdf</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>14</v>
+      </c>
+      <c r="E8" t="n">
+        <v>13</v>
+      </c>
+      <c r="F8" t="n">
+        <v>14</v>
+      </c>
+      <c r="G8" t="n">
+        <v>12</v>
+      </c>
+      <c r="H8" t="n">
+        <v>8</v>
+      </c>
+      <c r="I8" t="n">
+        <v>61</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Optimize</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>The biggest weakness is thin substance — the eBook reads as a high-level blog post rather than a gated asset with frameworks, data, or worked examples that justify a form fill; the product section also names the access control product 'Genea Security' which may not reflect current product naming (the help center references it as 'Genea' platform broadly, and brand positioning has evolved toward 'Genea Access Control' / cloud-native framing). The biggest strength is a clear, logical narrative arc that a rep can follow and that maps directly to real property-management pain points.</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>- Replace the thin 'Genea's Software Solutions' product blurb with a concrete before/after workflow example for at least one product (e.g., a step-by-step of how an on-demand HVAC request flows from tenant submission through automated billing to accounting integration), giving readers — and the rep — something substantive to reference in a deal conversation rather than a bullet list they could find on the website.
+- Verify and update the access control product name throughout: the document calls it 'Genea Security,' but current Genea positioning and help center materials refer to the access control offering without that label — align the name to whatever is live on getgenea.com today to avoid confusing a prospect mid-deal or embarrassing a rep.
+- Add a dedicated, designed call-to-action page at the end of the PDF itself (not just contact details in a footer) — the current closer is a list of phone/email/address with no directional language; replace or supplement it with a single, explicit next step such as 'Schedule a 30-minute workflow audit with a Genea specialist at getgenea.com/demo' so the asset can stand alone when forwarded by a prospect internally.
+- Introduce at least one concrete data point or customer proof — even an anonymized example (e.g., 'a 10-building portfolio reduced HVAC billing reconciliation from 8 hours/month to under 1 hour') — to give the 'biggest time sinks' section credibility and give the rep a quotable figure; right now all claims are asserted without evidence, which weakens the asset's ability to move a skeptical stakeholder.
+- Remove or update the physical mailing address and phone number from the contact footer and replace with a QR code or UTM-tagged URL so marketing can track PDF engagement and reps can send a clean digital version without outdated contact details creating support or routing confusion.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/genea-and-building-management-systems/</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Genea and Building Management Systems</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>STALE -- only copy found anywhere in SharePoint is from 2019 (Marketing/ALL MARKETING ARCHIVE/zArchived Marketing). No current version exists. Confirmed with Sarah as a known stale asset.</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>8</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>22</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>This asset is confirmed stale from 2019 and archived — it references an outdated data center compliance standard (SSAE-16, superseded by SSAE-18/SOC 2 Type II), a 128-bit VPN encryption claim that is below current industry norms, an old domain/contact format (getgenea.com with a 714 phone number that may be dead), and zero mention of Genea's current physical access control / security platform positioning. Its one strength is the technical depth on BMS protocol support, which remains a genuinely useful reference if verified and updated.</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>- Replace or retire this asset immediately before any rep accidentally attaches it to a deal — the SharePoint archive flag and Sarah's confirmation of staleness mean it should be unpublished from all sales enablement libraries as the highest-priority action; a placeholder one-pager with current BMS integration talking points is preferable to sending this.
+- Update the security compliance claims from SSAE-16 (retired in 2017) to current certifications (SOC 2 Type II at minimum) and upgrade the encryption claim from '128-bit VPN tunnel' to reflect current standards (AES-256 or equivalent), as these are the figures a security-conscious prospect or their IT team will immediately scrutinize.
+- Reposition the document around Genea's current cloud-native physical access control platform rather than leading with an HVAC/overtime BMS framing — the 2019 version predates the Security Platform product line entirely, and the help center reference articles (2N Intercom, Zenitel, Raptor, Triton integrations) demonstrate how much broader the integration story is today, none of which appear here.
+- Add a concrete next-step call to action inside the document body — currently there is no CTA whatsoever, not even a website URL prompt; at minimum add a 'Schedule a Technical Demo' or 'Contact your Genea rep' line with a current URL and contact path.
+- Audit and update the supported/not-supported BMS hardware lists against current engineering specs before republishing — five-year-old compatibility tables (e.g., Siemens Desigo listing, JCI Metasys DDE) may reflect discontinued firmware versions or newly supported systems, and a wrong 'NOT SUPPORTED' call sent to a prospect could kill a deal.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/genea-and-different-mechanical-setups/</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Genea and Different Mechanical Systems</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/archive/ebook, Case Studies, Whitepapers, One sheets/2024/one sheets/Genea &amp; Different Mechanical Systems.pdf (newest copy: 2023-24, still an archive-labeled folder)</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" t="n">
+        <v>13</v>
+      </c>
+      <c r="F10" t="n">
+        <v>14</v>
+      </c>
+      <c r="G10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>57</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>The biggest weakness is that this one-sheet is extremely thin — it reads as a simple FAQ with no data, customer examples, or frameworks to justify gating, and it completely lacks any call to action inside the document itself. Its biggest strength is that the core technical claims about BMS integration and hardware-agnostic compatibility appear accurate and consistent with Genea's current positioning.</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>- Add a concrete next-step CTA inside the document body (e.g., 'Schedule a 30-minute BMS compatibility review with a Genea solutions engineer at getgenea.com/demo') — the document currently ends abruptly with a list of mechanical system types and contains zero guidance on where the reader should go next, making it a dead end for any deal.
+- Upgrade the substance to justify gating: replace or supplement the FAQ format with at least one worked example or customer story (e.g., a commercial office building that reduced after-hours HVAC cost by X% using Genea's VAV-level control), since a plain Q&amp;A list offers nothing a prospect couldn't get from a chatbot or product page.
+- Reconcile the document's identity — the file is titled 'Genea and Different Mechanical Systems' but the header reads 'Overtime HVAC and Different Mechanical Systems,' creating brand confusion; standardize to the current product naming convention used across Genea's site and help center (the help center articles consistently use 'Genea' as the top-level brand with product lines named beneath it).
+- Expand the 'What if not all of my equipment is controlled by my BMS?' answer to describe the actual dual-path workflow in more detail (automated BMS path vs. manual Building Engineer email path), since this is a real differentiator that prospects with mixed-control environments will care about and currently the one-sentence answer undersells it.
+- Note in the document that the help center references provided cover access control integrations (ASSA ABLOY, Meraki, Schindler, Atrium) that are not mentioned here — if this one-sheet is handed to a prospect evaluating Genea holistically, a sidebar or footer callout linking to Genea's integration ecosystem would reinforce the 'hardware agnostic' claim with credible, named examples rather than leaving it as an assertion.</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/physical-access-control/</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Getting Started with Physical Access Control</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/eBooks/eBook - Physical Access Control.pdf</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>13</v>
+      </c>
+      <c r="E11" t="n">
+        <v>12</v>
+      </c>
+      <c r="F11" t="n">
+        <v>13</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10</v>
+      </c>
+      <c r="H11" t="n">
+        <v>8</v>
+      </c>
+      <c r="I11" t="n">
+        <v>56</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>The document is thin, generic, and undersells Genea's actual integration ecosystem — it mentions only three identity-provider integrations (Okta, Active Directory, OneLogin) while the help center confirms live VMS integrations with Rhombus, Eagle Eye, Milestone, and Tyco Cloud, plus a Slack integration, none of which appear here. Its biggest strength is that the onboarding step flow and core hardware components section give a prospect a useful orientation framework, but the content is too shallow to justify a gated form fill.</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>- Add a dedicated integrations section covering Genea's VMS partners (Rhombus, Eagle Eye, Milestone, Tyco Cloud) and Slack — all confirmed in current help center articles — because the document currently implies Genea's only integrations are three identity providers, which will cause a rep to look uninformed in front of any prospect who asks about video surveillance unification.
+- Expand the 'About Genea' and onboarding sections with at least one concrete, worked example or customer scenario (e.g., a multi-tenant office building replacing a legacy keycard system) to justify gating this behind a lead-capture form — right now the content is shorter and less specific than a typical blog post.
+- Replace the sparse 'About Genea' bullet list (intuitive, open, accountable, responsive) with specific, differentiated proof points tied to Genea's cloud-native, hardware-agnostic positioning — the current adjectives are generic and give a rep nothing to anchor a conversation to.
+- Add an explicit, on-page call to action at the end of the document (e.g., 'Schedule a free site survey at getgenea.com' or 'Contact your Genea rep to start Step 1') — the guide describes a five-step onboarding process but never tells the reader how to initiate it.
+- Audit and update the credential-type list to lead with mobile/NFC/BLE credentials rather than burying them, and explicitly name Genea's mobile credential offering if one exists, so the document reflects current market positioning rather than a hardware-first framing.</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/how-to-select-a-physical-security-platform-for-educational-institutions/</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>How to Select a Physical Security Platform for Educational Institutions</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Sales2/SALES Main Folder/Content/Whitepapers/Education Whitepaper.pdf (Genea-branded version, per Sarah's direction over the co-branded Carahsoft copy)</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" t="n">
+        <v>13</v>
+      </c>
+      <c r="F12" t="n">
+        <v>11</v>
+      </c>
+      <c r="G12" t="n">
+        <v>8</v>
+      </c>
+      <c r="H12" t="n">
+        <v>5</v>
+      </c>
+      <c r="I12" t="n">
+        <v>49</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>The document is dangerously thin — it reads as a checklist skeleton rather than a whitepaper, offering no worked examples, no data, no customer proof, and no meaningful narrative depth that would justify a form fill; the biggest strength is that its checklist topics (non-proprietary hardware, cloud, mobile credentials, integrations) do align directionally with Genea's core positioning, but none are developed enough to be credible or differentiated.</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>- Expand the integration section with specific, named integration partners that Genea actually supports today — the help center confirms live integrations with Eagle Eye, Tyco Cloud, Rhombus, Schlage AD/Engage series, and ASSA ABLOY Aperio series; naming even two or three of these in the education context (e.g., wireless Schlage locks on classroom doors, video verification via Rhombus) would immediately make the document concrete, accurate, and differentiated instead of generic.
+- Replace the bare bullet-point checklist format with at least one developed narrative section — a worked scenario such as 'a mid-size K-12 district migrating from a legacy proprietary system' with actual decision criteria, tradeoffs, and outcomes would deliver the substance required to justify gating this behind a form and give a rep a reason to send it over a free blog post.
+- Add a clear, dedicated call-to-action page or final section inside the PDF itself — the current closing line ('Now is the time to start research') is not a next step; replace it with a specific prompt such as 'Schedule a 30-minute demo with a Genea education specialist at getgenea.com/demo' so the document can stand alone when forwarded by a rep or printed.
+- Remove or reframe the 'Cloud-Based Access Control Security for 2025 and Beyond' header, which already reads as dated the moment 2025 arrives or passes; replace it with a forward-looking but evergreen frame (e.g., 'Built for How Schools Operate Today and Tomorrow') to prevent reps from having to apologize for stale language on a live deal.
+- Add a section specifically addressing student credential privacy and FERPA/state-privacy-law considerations — the document raises 'Issuing Credentials to Students' and 'assess privacy policy alignment' as a bullet but never addresses it, which is precisely the concern a university IT or legal stakeholder will raise and where a knowledgeable whitepaper could build real credibility.</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/implementing-touchless-access-control-into-your-building/</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Implementing Touchless Access Control into Your Building</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/eBooks/eBook - Implementing Touchless Access into Your Building.pdf</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>7</v>
+      </c>
+      <c r="E13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F13" t="n">
+        <v>8</v>
+      </c>
+      <c r="G13" t="n">
+        <v>11</v>
+      </c>
+      <c r="H13" t="n">
+        <v>5</v>
+      </c>
+      <c r="I13" t="n">
+        <v>41</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>The document is heavily anchored in COVID-era concerns (PPE mandates, sick-stay-home policies, thermal cameras, staggered start times) that read as deeply dated for a prospect in 2024-2025, undermining credibility the moment a rep attaches it to a deal. Its strongest element is the structured breakdown of touchless access layers (mobile, elevator, door hardware, cloud management), which provides a legitimate framework — but that framework needs to be decoupled from pandemic framing and updated with current product details.</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>- Remove or fully reframe all COVID-specific content — including the PPE mandates, sick-stay-home procedural guidance, thermal camera section, and staggered-schedule recommendations — as these read as a 2020 artifact and will immediately erode prospect confidence in Genea's currency; replace with a modern physical security threat framing (tailgating, hybrid workforce credential sprawl, multi-site portfolio management) that makes the touchless case without pandemic dependency.
+- Replace the vague 'Touchless Elevators' section (which describes only generic relay-based and hand-wave actuators) with Genea's actual, named destination dispatch integrations: per the help articles 'Genea Access Control System Integration with KONE Destination Dispatch Elevator System' and 'Genea Access Control System Integration with Mitsubishi Destination Dispatch Elevator System,' Genea supports specific hardware (KONE D820/D880 via Genea gateway, Mitsubishi via Mercury LP4502/MP4502 controllers) — naming these gives a rep concrete proof points and differentiates from a generic whitepaper.
+- Reconcile the customer retention stat: the opening pull-quote says '99% customer retention' but the stat block immediately below it says '98% Customer Retention' — a rep sending this to a prospect will be asked about the discrepancy and has no clean answer; pick one figure (the current, defensible number) and make it consistent throughout.
+- Add a concrete next-step CTA inside the document itself — the content ends with a key-takeaways list and a product name drop ('Genea Security, On-Demand HVAC, Submeter Billing') but includes no request-a-demo link, no QR code, no contact prompt, and no suggested follow-on resource; a single closing page with a demo URL and one-line description of what a Genea demo covers would directly address the lowest-scoring dimension.
+- Update the product suite listing to reflect current Genea branding and positioning — 'Genea Security, On-Demand HVAC, Submeter Billing' is a flat product list with no cloud-native or non-proprietary-hardware messaging; this is the one place in the document where Genea's differentiated brand story should land, and it currently reads like a nav menu; rewrite it as two to three benefit-led sentences that connect the touchless access argument made in the body to the broader smart-building platform.</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/submeters-101/</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Learn the Facts - Submeters 101</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/Whitepapers/Submetering 101 - Whitepaper.pdf</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>14</v>
+      </c>
+      <c r="E14" t="n">
+        <v>13</v>
+      </c>
+      <c r="F14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H14" t="n">
+        <v>6</v>
+      </c>
+      <c r="I14" t="n">
+        <v>53</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>The document is extremely thin — four short paragraphs that read more like a landing-page blurb than a whitepaper — and fails to surface any of the product's actual capabilities (mobile app, QR-code commissioning, portal-based statement distribution, audit workflow) that the help center confirms exist today; the biggest strength is that the core educational framing (master meter → proration problem → submeter solution) is accurate and a reasonable hook for a cold prospect.</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>- Expand the 'How Does It Work?' section to describe Genea's actual networked-meter workflow end-to-end — QR-code commissioning via the mobile app, automated read uploads, Genea billing-team audit, Property Manager approval, and tenant portal statement access — all of which are confirmed in the help center articles 'How to commission a meter,' 'Getting started with Genea's Submeter Billing Mobile App,' and 'How to Access Tenant Metering Statements'; this is the single biggest gap between what the document promises and what the product actually delivers.
+- Add a dedicated section on the three statement types (Building Summary, Tenant Summary, Meter Detail) using the structure confirmed in the help article 'How to Read Metering Statements,' so a prospect understands the reporting artifact they will actually receive — this directly counters the vague 'professional monthly invoices' claim and gives the asset gatable substance.
+- Replace the generic closing paragraph ('Genea's meter reading and billing service takes the hassle out of submetering') with a specific, visible call to action inside the PDF — e.g., 'Schedule a demo at getgenea.com/demo' or a named sales contact — since the document currently has no next-step directive for a reader who received it directly from a rep.
+- Reframe the 'WHY SUBMETER?' bullet list into a before/after narrative or a brief ROI framework (e.g., time saved on manual reads, invoice dispute reduction) to justify the lead-gate friction; four undifferentiated bullets about carbon footprint awareness do not deliver the depth a prospect expects from a whitepaper versus a blog post.
+- Add a 'Who This Is For' scope line near the top (property manager, tenant, building engineer) and call out the mobile app's iOS/Android availability and push-notification feature for pending uploads (per the help article 'Meter Read Upload Notifications') so a rep can confidently send this to a specific persona without caveating the relevance.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/submeters-102/</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Learn the Facts - Submeters 102</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/Whitepapers/Submetering 102 - Whitepaper.pdf</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>14</v>
+      </c>
+      <c r="E15" t="n">
+        <v>13</v>
+      </c>
+      <c r="F15" t="n">
+        <v>13</v>
+      </c>
+      <c r="G15" t="n">
+        <v>12</v>
+      </c>
+      <c r="H15" t="n">
+        <v>4</v>
+      </c>
+      <c r="I15" t="n">
+        <v>56</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>The document's biggest weakness is a near-total absence of a next-step call to action — it ends abruptly with a use-case bullet and gives the reader nowhere to go — compounded by thin, blog-level content that doesn't justify a gate. Its biggest strength is accurate, practical coverage of meter types and data-collection methods that a property manager would find genuinely useful as a starting framework.</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>- Add a specific, in-document CTA at the close — at minimum a sentence such as 'Schedule a demo with a Genea submetering specialist at getgenea.com/demo' — because the document currently ends on a technical bullet with zero guidance on next steps, making it a dead end for every rep who attaches it to a deal email.
+- Integrate Genea's Submeter Billing Mobile App (per the help article 'Getting started with Genea's Submeter Billing Mobile App') as a named, described feature in the 'Collecting Data' section — the whitepaper mentions 'a recording service like Genea' but never names or explains the mobile app, missing a direct product proof point that differentiates Genea from generic pulse-output services.
+- Expand 'Using the Data' from a four-item bullet list into at least one worked example or mini case study (e.g., a hypothetical 200,000 sq ft office building recovering $X in utility costs after 90 days of submetering) so the content earns its gate — currently this section is shallower than a typical blog post and a prospect who fills out a form will feel shortchanged.
+- Update the meter brand references (Dent PowerScout, Triacta, Emon Dmon Class 3400) with a note on current Genea-certified or Genea-integrated hardware to avoid a rep having to apologize if a prospect asks 'does Genea still work with these?' and the answer has changed.
+- Add a dated 'Last reviewed' line to the footer or cover page so reps and prospects can immediately assess currency — the document carries no publication or revision date, which erodes trust when shared in a live deal context.</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/nycs-local-law-97-a-guide-for-real-estate-teams-adopting-sustainability-solutions/</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>NYC's Local Law 97: A Guide for Real Estate Teams</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Sales2/SALES Main Folder/Content/Whitepapers/CRE/Whitepaper - NYC's Local Law 97.pdf</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>14</v>
+      </c>
+      <c r="E16" t="n">
+        <v>15</v>
+      </c>
+      <c r="F16" t="n">
+        <v>14</v>
+      </c>
+      <c r="G16" t="n">
+        <v>11</v>
+      </c>
+      <c r="H16" t="n">
+        <v>7</v>
+      </c>
+      <c r="I16" t="n">
+        <v>61</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>The biggest weakness is thin substance — the document reads as a one-page marketing flyer rather than a gated whitepaper, with no data sources cited, no worked financial example, and no meaningful compliance framework beyond a four-bullet checklist that a prospect could find on any NYC government page; the biggest strength is that the core product positioning (On-Demand HVAC as a LL97 compliance lever, 40% runtime reduction claim, hybrid-work angle) is coherent and differentiated.</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>- Replace the vague 'reducing HVAC runtime by 40% on low occupancy days' claim with a sourced customer case study or methodology footnote — an unsupported statistic in a gated asset actively damages credibility with the facilities directors and ESG officers most likely to read it, and without sourcing a rep cannot defend it in a follow-up meeting.
+- Expand the 'Checklist: How to Comply' section into a genuine compliance framework: map each checklist step to the specific LL97 penalty calculation formula ($/metric ton of CO2 above limit), show a worked example building (e.g., 100,000 sq ft office at 5.2 kg CO2/sq ft), and quantify where On-Demand HVAC impacts the calculation — this is the substance that justifies a form fill and differentiates the asset from free NYC DOB guidance.
+- Add a concrete next-step call to action inside the document body (not just a footer URL) — the current closing line 'Don't Get Caught Paying Fines' ends on a threat with no directed action; replace or follow it with a specific offer such as 'Schedule a 30-minute LL97 impact assessment with a Genea engineer at getgenea.com/demo' to give sales reps a trackable handoff point.
+- Per the help articles 'How do I access Genea Overtime HVAC service?' and 'Creating an Overtime HVAC Request via a Mobile app,' the product is consistently named 'Overtime HVAC' in current product documentation, yet this whitepaper uses 'On-Demand HVAC' throughout — reconcile the naming to whichever is the current go-to-market label so reps are not handing prospects a document that conflicts with the product UI and support portal they will actually use.
+- Cite the 2024 compliance deadline and the 2030 / 2050 penalty tier structure with a reference to the official NYC Local Law 97 text or a dated source, and note whether the 2024 enforcement start date has already passed (it has) — framing the law as a future event when fines are already accruing makes the asset read as stale and could embarrass a rep sending it mid-deal in 2025.</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/overtime-hvac-and-real-life-scenarios/</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>On-Demand HVAC and Real Life Scenarios</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/eBooks/eBook- ODHVAC Real Life Scenarios.pdf (original Whitepapers-folder PDF failed text extraction -- image-heavy/scanned; this is an alternate eBook copy of the same asset)</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>15</v>
+      </c>
+      <c r="E17" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" t="n">
+        <v>13</v>
+      </c>
+      <c r="G17" t="n">
+        <v>10</v>
+      </c>
+      <c r="H17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" t="n">
+        <v>57</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>The biggest weakness is severe thinness: the content is essentially a bulleted feature glossary with no worked examples, data, customer stories, or frameworks despite promising 'real life scenarios' in the title — the asset does not deliver what it advertises and lacks any closing CTA. Its biggest strength is accurate feature coverage; every capability listed (minimum run time, split billing, tiered billing, courtesy start, etc.) aligns with how the help center describes the OD HVAC product and no deprecated or contradictory claims were found.</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>- Add at least two or three concrete 'real life scenario' narratives (e.g., a multi-floor law firm using tiered billing + recurring requests for Friday evening partner meetings, or a property manager using courtesy start + minimum bill time for a weekend tenant) — the title explicitly promises these and the asset currently delivers none, which will disappoint any prospect who fills out a form expecting worked examples.
+- Replace the plain bullet list structure with a visual or tabular format that maps each scenario/feature to a specific tenant or property-manager pain point (e.g., 'Problem: tenant complains room is still cold at the requested start time → Solution: Courtesy Start'), giving the asset the depth needed to justify a form fill over a public blog post.
+- Add a closing call-to-action section directing the reader to schedule a demo or contact their Genea rep — the document ends abruptly after 'Double Billing' with zero next-step guidance, leaving a rep with nothing to point the prospect toward.
+- Rename or reframe the 'Lease Hours Only Users' bullet to align with the exact role label used in the help center article 'Managing Users in the OD HVAC Portal,' which calls this role 'Lease Only Tenant User' — the current phrasing ('LEASE HOURS ONLY USERS') is close but inconsistent and could confuse prospects comparing the doc to the portal UI.
+- Add a brief introductory paragraph or one-sentence context line for each feature cluster (billing rules, user controls, scheduling) so a rep can hand this to a property manager or asset manager who is unfamiliar with on-demand HVAC concepts without needing to verbally explain the structure of the document.</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/passing-through-the-cost-of-your-overtime-hvac-software-to-your-tenants/</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Passing Through the Cost of On-Demand HVAC Software to Tenants</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/archive/archive/Passing Through the Cost of Overtime HVAC Software to Your Tenants.pdf</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>13</v>
+      </c>
+      <c r="E18" t="n">
+        <v>12</v>
+      </c>
+      <c r="F18" t="n">
+        <v>14</v>
+      </c>
+      <c r="G18" t="n">
+        <v>13</v>
+      </c>
+      <c r="H18" t="n">
+        <v>6</v>
+      </c>
+      <c r="I18" t="n">
+        <v>58</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>The biggest issue is the complete absence of a next-step call to action inside the document itself, leaving a converted prospect with nowhere to go; the biggest strength is the worked cost-passthrough example, which is a genuinely useful financial framework that justifies the gate and directly addresses a real objection for property managers.</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>- Add a closing CTA section — at minimum one sentence with a link or instruction (e.g., 'Schedule a demo at getgenea.com/demo to see how Genea's On Demand HVAC portal automates requests and invoicing for your building') — since the document currently ends with no prompt for next steps, making it a dead end for a prospect who has already converted.
+- Reconcile the product naming throughout: the help center articles (e.g., 'Managing Users in the OD HVAC Portal' and 'How do I access Genea Overtime HVAC service?') use both 'Overtime HVAC' and 'On Demand HVAC' interchangeably, and the document's own title switches between 'On-Demand HVAC' (cover/filename) and 'Overtime HVAC' (body) — pick one name and apply it consistently, or explicitly explain that On Demand is the current product name if a rebrand has occurred.
+- Update the 'Genea ACS Cloud' line item label visible in the costing spreadsheet description — this legacy product name does not appear in any current help center documentation and may confuse prospects or require a rep to explain outdated nomenclature mid-deal.
+- Expand the substance beyond the single cost-passthrough angle by adding one concrete tenant or property outcome (e.g., a quoted average uplift in after-hours HVAC revenue, or a brief anonymized building example) so the asset delivers differentiated proof a prospect could not get from a blog post or a one-paragraph web page.
+- Remove or update the '© 2023' copyright date on the cover, which signals to a prospect reviewing this in 2024 or 2025 that the material may be stale, undermining confidence in the figures cited.</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Quick Win</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/proprietary-vs-open-hardware/</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Proprietary vs. Open Hardware</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/Whitepapers/Proprietary vs. Open Hardware.pdf</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>13</v>
+      </c>
+      <c r="E19" t="n">
+        <v>12</v>
+      </c>
+      <c r="F19" t="n">
+        <v>11</v>
+      </c>
+      <c r="G19" t="n">
+        <v>9</v>
+      </c>
+      <c r="H19" t="n">
+        <v>8</v>
+      </c>
+      <c r="I19" t="n">
+        <v>53</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>The biggest strength is the core Mercury-based open-hardware argument, which is directionally correct and supported by the help center reference on Mercury MP vs. LP series. The biggest issues are thinness of content (this reads as a one-page blog post, not a whitepaper or eBook worthy of a form fill), specific pricing figures ($250 readers, $850 controllers, $500 installation) that are undated and unattributed and will erode credibility with a savvy buyer, and the combative 'You're Being Deceived' framing that puts a rep in an awkward position when sending to a prospect.</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>- Replace or substantiate the hardware cost figures (20 x $250 readers, 4 x $850 controllers, 20 x $500 installation) with either a sourced, dated estimate or a range with a footnote — a procurement-literate prospect will immediately question unattributed unit prices, and a rep has no way to defend them if challenged.
+- Expand the content to genuine whitepaper depth: the current text is roughly 250 words and fits on one page, which does not justify a gated lead-capture form; add sections on total cost of ownership methodology, migration risk frameworks, or a second worked example with a different building profile to deliver value a prospect cannot get from a blog post.
+- Soften the opening 'You're Being Deceived' headline and the closing 'don't be fooled by marketing gimmicks' line — this adversarial tone can embarrass a rep sending the asset directly to a prospect or a facilities director at an enterprise account; replace with confident, evidence-led framing such as 'How to Evaluate Open vs. Proprietary Access Control Hardware.'
+- Per the help article 'Mercury MP series versus LP series,' the document's claim that Mercury controllers have been 'used by over two dozen access control software companies since the 90s' is consistent with the reference but the whitepaper omits the current Mercury product line distinction (MP vs. LP series) that a technical buyer will ask about — add a brief note clarifying which Mercury series Genea supports to preempt that objection.
+- Add a structured, in-document next step beyond the single closing sentence — for example, a shaded call-out box with 'Schedule a Demo,' a QR code, or a reference to a related Genea resource on visitor management integration — so the asset can stand alone when printed or forwarded without the landing page context.</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/quantifying-the-value-of-your-after-hours-hvac-program/</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Quantifying the Value of Your After Hours HVAC Program</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/archive/archive/Quantifying the Value of Your After Hours HVAC Program.pdf</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>15</v>
+      </c>
+      <c r="E20" t="n">
+        <v>14</v>
+      </c>
+      <c r="F20" t="n">
+        <v>13</v>
+      </c>
+      <c r="G20" t="n">
+        <v>10</v>
+      </c>
+      <c r="H20" t="n">
+        <v>6</v>
+      </c>
+      <c r="I20" t="n">
+        <v>58</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>The document's biggest weakness is its extreme thinness — it reads as a one-page internal framework slide dressed up as an eBook, not a substantive gated asset, and the only concrete next step ('a complete case study available on request') is vague and passive. Its biggest strength is that the four-value-driver framework is genuinely relevant and strategically sound for a CRE audience evaluating an HVAC automation investment.</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>- Replace the placeholder 'case study available on request' line with an actual embedded or appended case study with named building type, quantified results (e.g., % billing leakage recovered, hours saved per month), and a direct CTA to schedule a demo at getgenea.com/demo — this single change would simultaneously fix the substance gap and the next-step gap, the two lowest-scoring areas.
+- Expand the Energy Savings section to reflect the product's actual workflow as documented in the help articles: specifically, the Genea Portal (portal.getgenea.com) and mobile app enable tenants to self-serve requests, which means occupancy data can be captured digitally — explain how this closes the gap between assumed and actual occupancy rather than pointing prospects back to manual 'access card log' checks, which undersells the automation.
+- Add at least one worked numeric example per value driver (e.g., '50 after-hours requests/month × 20 min/request × $35/hr = $583/month in labor alone') so the 'quantifying' promise of the title is actually delivered in the body of the document, not just described as a methodology.
+- Update the product naming throughout to consistently use 'On Demand HVAC' (the current portal label per the help article 'Managing Users in the OD HVAC Portal') rather than the generic 'after-hours HVAC program' or 'overtime HVAC workflow' — inconsistent naming creates friction when a rep's demo environment shows 'OD HVAC Portal' and the asset uses different language.
+- Add a visible, specific closing CTA inside the document itself — e.g., a designed end-page with 'See how [Building Type] recovered $X in billing leakage — book a 20-minute demo at getgenea.com/demo' — so the asset can stand alone when a rep forwards the PDF directly without the landing page context.</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/safe-workplace/</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Safe Workplace</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>AllEmployees2/General/2022 Collateral/Safe Workplace.pdf</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>8</v>
+      </c>
+      <c r="E21" t="n">
+        <v>10</v>
+      </c>
+      <c r="F21" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" t="n">
+        <v>7</v>
+      </c>
+      <c r="H21" t="n">
+        <v>3</v>
+      </c>
+      <c r="I21" t="n">
+        <v>34</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>This asset is a 2022 COVID-era one-pager whose entire premise — capacity limits, health questionnaires, contact tracing, and body-temperature-scanner integrations — is anchored in pandemic-era use cases that are no longer a credible sales motion for most prospects today; a rep attaching this to a live deal risks looking out of touch or raising uncomfortable questions about product direction. The one strength is that the core feature set described (mobile check-in, capacity alerts, admin-approval workflows, registration cards) does appear to still exist in the current help center docs, so the feature itself has not been deprecated outright.</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>- Remove or completely reframe all COVID-19 / pandemic-era language and the body-temperature-scanner integration bullet — the help center article 'About Genea's Safe Workplace Feature' itself frames this feature as a coronavirus response, and leading with that framing in a current sales asset will immediately date the document and undermine rep credibility in any post-2023 deal.
+- Add a clear call-to-action inside the document (e.g., 'Schedule a demo' with a URL or QR code, or a 'Talk to sales' prompt) — the document currently ends with a feature bullet list and has no next-step guidance whatsoever, meaning a prospect who reads it has nowhere to go without the rep following up manually.
+- Reposition the use cases around modern, evergreen workplace scenarios — hybrid office management, compliance with building occupancy codes, visitor credentialing, or enterprise security policy enforcement — rather than pandemic return-to-office, so the asset can survive more than one selling season.
+- Expand thin feature bullets into brief outcome statements with at least one quantified example or customer reference (e.g., 'reduced manual check-in overhead by X%' or a named customer quote), since the current one-page bullet list does not justify the friction of a gated form fill for a prospect who already converted.
+- Update the copyright line from '© Genea 2022' and verify the getgenea.com URL and any implied links are still active, as stale copyright years and dead links are the first thing a skeptical enterprise buyer notices and they signal neglect of the asset library.</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/safeguard-the-workplace-during-and-beyond-the-covid-19-pandemic/</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Safeguard the Workplace During and Beyond COVID-19</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>AllEmployees2/2023 Collateral/eBooks/Access Control/eBook- Occupancy Management.pdf (renamed at some point from its original title -- content confirms it's the same asset)</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>7</v>
+      </c>
+      <c r="E22" t="n">
+        <v>10</v>
+      </c>
+      <c r="F22" t="n">
+        <v>5</v>
+      </c>
+      <c r="G22" t="n">
+        <v>8</v>
+      </c>
+      <c r="H22" t="n">
+        <v>4</v>
+      </c>
+      <c r="I22" t="n">
+        <v>34</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>The single biggest issue is that the entire asset is built around COVID-19 pandemic-era use cases (health questionnaires, thermal sensors, social distancing thresholds) that are functionally obsolete and would embarrass a rep attaching this to any deal today; the biggest strength is that the core Safe Workplace feature set it describes does appear to match actual current product capabilities per the help center references, so the underlying product content could be salvaged into a modernized occupancy-management or workplace-intelligence narrative.</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>- Replace the COVID-19 framing entirely — retitle and restructure the asset around evergreen occupancy management, space utilization, and compliance use cases (e.g., lease right-sizing, fire-code compliance, hybrid workforce planning); the help center articles confirm Safe Workplace's capacity, contact-tracing, and screening features still exist, but the pandemic rationale for using them is no longer a credible sales hook for most prospects in 2024+.
+- Remove or recontextualize the thermal-sensor and 'social distancing' capacity-reduction copy ('reduce capacity from 100 to 20 with a single keystroke' framed as a COVID measure) — these read as dated product artifacts; per the help article 'Setting Capacity Restrictions for Your Property,' the capacity feature is real and current, so reframe it around operational density control and building-code compliance rather than pandemic response.
+- Add a concrete next-step call to action inside the document itself — the asset ends with product differentiators but contains no demo link, contact prompt, QR code, or 'talk to a rep' instruction; a rep cannot send this without manually appending context, which kills confidence in the asset.
+- Verify and update the 'three flagship product offerings' claim (Submeter Billing, Overtime HVAC, Access Control) against current Genea product packaging — if Safe Workplace is now a named module or if product naming has changed, this list either under-sells the portfolio or uses stale nomenclature that could create confusion mid-deal.
+- Add at least one concrete customer outcome, benchmark, or worked example (e.g., 'a 200,000 sq ft multi-tenant building reduced manual check-in overhead by X%') to justify gating this behind a lead-capture form; the current asset reads as a feature list that a prospect could extract from the public website.</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/the-3-essential-characteristics-of-access-control-for-integrators/</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>The 3 Essential Characteristics of Access Control</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Sales2/SALES Main Folder/Content/Whitepapers/Whitepaper - The 3 Essential Characteristics of Access Control.pdf</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>13</v>
+      </c>
+      <c r="E23" t="n">
+        <v>14</v>
+      </c>
+      <c r="F23" t="n">
+        <v>13</v>
+      </c>
+      <c r="G23" t="n">
+        <v>9</v>
+      </c>
+      <c r="H23" t="n">
+        <v>5</v>
+      </c>
+      <c r="I23" t="n">
+        <v>54</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>The document is dangerously thin for a gated asset — it reads more like a one-page leave-behind than a whitepaper, with almost no frameworks, data depth, or worked examples beyond a single customer quote; the 2022 market-sizing stat is the only data point and is now visibly dated, which undermines credibility with a sophisticated prospect reviewing it today.</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>- Replace the 2022 Research and Markets figure with a current (2024/2025) ACaaS market-size citation, or remove it entirely — a two-year-old valuation number in a gated document signals stale content to any procurement-savvy reader and is the single fastest credibility killer to fix.
+- Expand the VMS integration list and language to reflect the full current integration ecosystem confirmed in the help center: the document names Meraki, Ava, Salient, and Rhombus but omits Tyco Cloud, Eagle Eye, and Milestone Kite — all of which have dedicated integration articles in the Genea help center — leaving the connectivity claim feeling narrower than reality.
+- Replace the generic closing CTA ('Visit www.getgenea.com') with a specific, friction-matched next step such as a direct demo-booking link or a 'Talk to a Genea expert' prompt with a named URL; the current CTA is the weakest possible ending for an asset a rep attaches to a live deal email.
+- Dramatically increase substance to justify the gate: add at least one concrete framework (e.g., a scored evaluation rubric for assessing ACaaS readiness across the three characteristics), one additional customer example with quantified outcome, and a comparison table of proprietary vs. non-proprietary hardware tradeoffs — without these, a prospect who fills out a form will feel under-rewarded and a rep will hesitate to send it to a mid-funnel enterprise contact.
+- Rename or reframe 'Emergency Door Plans' to match current product terminology — per the help center article 'Creating and managing custom roles in Genea,' the feature surface around emergency plans is referenced as 'emergency plans' within the permissions/control-center context; verify current product naming in the UI and update the whitepaper to match so reps are not fielding questions about a feature name that doesn't appear in the product.</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/the-four-most-common-submeter-billing-mistakes/</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>The Four Most Common Submeter Billing Mistakes</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/archive/archive/The Four Most Common Submeter Billing Mistakes.pdf</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>14</v>
+      </c>
+      <c r="E24" t="n">
+        <v>13</v>
+      </c>
+      <c r="F24" t="n">
+        <v>14</v>
+      </c>
+      <c r="G24" t="n">
+        <v>10</v>
+      </c>
+      <c r="H24" t="n">
+        <v>8</v>
+      </c>
+      <c r="I24" t="n">
+        <v>59</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>The biggest weakness is thinness: this is a short list-format piece that doesn't justify a gate — it reads like a blog post or a leave-behind one-pager, not a substantive eBook a prospect would trade their contact info for. The biggest strength is that the four mistake categories are genuinely accurate and relatable pain points for the target persona, and the content does not contradict the help center references.</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>- Expand the asset to deliver eBook-worthy depth: add worked dollar-loss examples for each mistake type (e.g., a realistic scenario showing how a mistyped multiplier of 12,000 vs. 1,200 produces a specific monthly billing error), frameworks for auditing an existing spreadsheet, or anonymized customer before/after data — the current version is too thin to earn a form fill and would likely disappoint a prospect who just converted.
+- Replace the vague 'Genea's Submeter Billing service automates billing' closing with a concrete description of the mobile app workflow — per the help articles 'Getting started with Genea's Submeter Billing Mobile App' and 'How to commission a meter?', the product uses QR-code-based meter commissioning and a mobile companion app to eliminate manual clipboard reads; surfacing this specific mechanism makes the solution claim credible rather than generic.
+- Add an explicit, designed call-to-action section at the end of the document (not just a sentence) that directs the reader to a next step — e.g., 'Request your free spreadsheet audit' with a URL or contact path, and/or 'Book a 20-minute demo'; the current closing buries the free audit offer in plain body text with no visual emphasis or link, making it easy to miss.
+- Update the copyright year from 2023 and audit for any implicit staleness — if this asset is being handed to prospects in 2025 a two-year-old date on a document a rep attaches to a deal email signals neglect and may prompt a prospect to question whether the product information is current.
+- Add a section or callout explaining how Genea handles the rollover and multiplier problems specifically at the platform level (e.g., does the mobile app warn on out-of-range readings per the FAQ article 'Why am I seeing a meter reading range warning?') — this closes the logical gap between 'here are scary mistakes' and 'here is exactly how Genea prevents each one,' which is the persuasive move the asset currently skips.</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/access-control-guide-to-opening-a-new-office/</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>The Ultimate Access Control Guide to Opening a New Office</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/eBooks/eBook - Guide to Opening a New Office.pdf</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>14</v>
+      </c>
+      <c r="E25" t="n">
+        <v>13</v>
+      </c>
+      <c r="F25" t="n">
+        <v>14</v>
+      </c>
+      <c r="G25" t="n">
+        <v>15</v>
+      </c>
+      <c r="H25" t="n">
+        <v>8</v>
+      </c>
+      <c r="I25" t="n">
+        <v>64</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Optimize</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>The biggest weakness is a thin, generic CTA at the close combined with an integrations list (Okta, Active Directory, OneLogin) that omits current hardware and video partners documented in the help center — Schlage, ASSA ABLOY Aperio, Tyco, Eagle Eye, OpenEye — making the asset feel narrower than Genea's actual ecosystem. The biggest strength is the practical, buyer-ready cost benchmarking and hardware/installation process breakdown, which delivers genuine utility for a prospect planning a new office buildout.</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>- Add a dedicated integrations section — or expand the 'About Genea' blurb — to call out Schlage AD/Engage, ASSA ABLOY Aperio, Tyco Cloud VMS, Eagle Eye, and OpenEye VMS by name; these are all documented in current help center articles and their absence makes Genea look like an identity-only play rather than a full physical-security platform.
+- Replace the vague closing paragraph with a specific, action-oriented CTA inside the PDF itself — e.g. 'Book a 30-minute walkthrough of Genea's access control platform at getgenea.com/demo' — because the document currently ends without directing the reader anywhere, leaving a rep with no anchor for follow-up.
+- Update the cost figures ($650/door installation, $800/door hardware) with a dated caveat or range qualifier (e.g. 'as of [year]; your integrator will provide a site-specific quote') so a rep is not put in the position of defending specific numbers that may have shifted with supply-chain and labor-cost changes since publication.
+- Reframe the visitor management section to explicitly name Genea's native visitor management app as a product feature — not just a generic capability — and tie it to the 'one central system' consolidation message that already appears in the asset, reinforcing the 'extend beyond the door' positioning Genea uses.
+- Expand the SAML SSO / automatic provisioning bullet into at least two sentences naming supported IdPs (Okta, Active Directory, OneLogin are already cited) and noting that mobile credentials with SSO reduce IT overhead at move-in — this is the proof point a security-conscious buyer or IT stakeholder will look for and it currently reads as a throwaway line.</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Quick Win</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/touchless-visitor-management/</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Touchless Visitor Management</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>AllEmployees2/2022 Collateral/Visitor Management.pdf (newest copy found: 2022 -- no more recent version located)</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" t="n">
+        <v>9</v>
+      </c>
+      <c r="F26" t="n">
+        <v>7</v>
+      </c>
+      <c r="G26" t="n">
+        <v>8</v>
+      </c>
+      <c r="H26" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" t="n">
+        <v>35</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>The document is materially stale: it is dated 2022, frames the product around 'post-Covid-19' and a 'COVID-19 questionnaire system' as primary selling points—language that will actively undermine credibility with a prospect today—and it omits current credential features (Scramble QR Codes, Neat Frame device support) documented in the help center. Its single biggest strength is that the core feature list (pre-registration, QR codes, multi-tenant, badge printing) still maps to real product capabilities, giving a refresh a solid foundation to build on.</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>- Replace all COVID-19 framing ('post-Covid-19 world,' 'COVID-19 questionnaire system,' 'COVID-19 health questions') with evergreen language about visitor security, compliance workflows, and customizable health or policy questionnaires—this language is the most damaging element a rep would have to apologize for in a live deal.
+- Add a section on Scramble QR Code badges: per the help article 'How to Utilize the Scramble QR Code Badge,' this is a distinct, newer credential type compatible with mobile web browsers that visitors access via a unique URL—its omission makes the document feel behind the current product.
+- Update the touchless check-in description to reflect that walk-in visitors can scan a QR code displayed on the iPad Kiosk or a printed lobby code (per 'Touchless Check-In for Walk-In Visitors'), and that Neat Frame devices are also supported as kiosk hardware (per 'How to Enable Pre-Registered Guest Check-In on the Kiosk App')—the document currently implies touchless is only for pre-registered guests arriving with a code.
+- Add a clear in-document call to action—currently the asset ends with a bare feature bullet list and no next step; at minimum add a closing section directing the reader to request a demo or contact their Genea rep, including a URL or email, so a rep doesn't have to append a manual note.
+- Expand the 'Advanced Features' bullet list into brief descriptive sentences or a short paragraph for at least three of the eight items (e.g., NDA/Document Signing, Native Multi-Tenant Support, Reporting and Analytics) to give the asset enough substance to justify a form fill over a product page scan.</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Quick Win</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>https://www.getgenea.com/downloads/understanding-the-differences-between-nfc-and-bluetooth/</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Understanding the Differences Between NFC and Bluetooth</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Marketing/CONTENT/Whitepapers/Whitepaper - Apple Wallet - NFC vs Bluetooth.pdf</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>13</v>
+      </c>
+      <c r="E27" t="n">
+        <v>13</v>
+      </c>
+      <c r="F27" t="n">
+        <v>12</v>
+      </c>
+      <c r="G27" t="n">
+        <v>10</v>
+      </c>
+      <c r="H27" t="n">
+        <v>4</v>
+      </c>
+      <c r="I27" t="n">
+        <v>52</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>The biggest weakness is that this document is extremely thin — it reads as a glossary/primer rather than a substantive gated asset, and it ends with no call to action whatsoever, making it nearly useless as a sales closer. Its biggest strength is the Apple Wallet + HID section, which correctly reflects current product capability and gives the document its only real differentiation.</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>- Add a call to action: the document currently ends mid-paragraph with no next step — insert a closing section directing the reader to request a demo or contact their Genea rep, consistent with how other gated assets close (e.g., 'See Genea mobile access in action — schedule a demo at getgenea.com').
+- Expand coverage of Google Wallet / Android NFC: the help article 'Add to Google Wallet - HID X Genea Mobile Access' confirms Genea supports Google Wallet with NFC for Android via HID readers, but the whitepaper mentions only Apple Wallet, making the document appear iOS-only and potentially alienating Android-heavy prospects or facility managers.
+- Replace the generic security comparison section with Genea-specific, decision-relevant content: the current 'Is Bluetooth Access Control More Secure?' section reads as a Wikipedia entry — reframe it around why Genea's implementation (App-Based BLE keys vs. Apple/Google Wallet NFC keys) was designed the way it is, using the two key types described in 'Genea Mobile App - iPhone User Guide' and 'Genea Mobile Access App - Android User Guide' as the concrete anchor.
+- Add a practical buyer framework or decision guide: the whitepaper promises to explain 'why NFC and BLE matter to mobile access control security' but never delivers a usable answer — add a simple table or scenario guide (e.g., high-traffic lobby = NFC tap speed advantage; long-range hands-free = BLE advantage) so a prospect or IT evaluator can map the technology choice to their environment, justifying the gate.
+- Audit and update the BLE specification claim: the document states BLE operates at '~1 MB/sec,' which overstates real-world BLE throughput (actual BLE 4.x air data rate is 1 Mbps but effective throughput is far lower); correct this to avoid credibility loss with a technically sophisticated buyer such as an IT director or security architect.</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Major Project</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>